<commit_message>
feat(db): clean participants tab in excel database template
</commit_message>
<xml_diff>
--- a/porra_mundial_db.xlsx
+++ b/porra_mundial_db.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,142 +433,6 @@
       <c r="C1" t="inlineStr">
         <is>
           <t>paid</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>p01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Carlos</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>p02</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>María</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>p03</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Javi</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>p04</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Laura</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>p05</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Pedro</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>p06</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Ana</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>p07</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Diego</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>p08</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Lucía</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>FALSE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(events): select E2 wild match randomly during database generation
</commit_message>
<xml_diff>
--- a/porra_mundial_db.xlsx
+++ b/porra_mundial_db.xlsx
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -23397,7 +23397,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>El administrador sortea un partido especial que dobla los puntos de las predicciones.</t>
+          <t>Un partido del mundial seleccionado aleatoriamente que otorga el doble de puntos.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -23408,10 +23408,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Partido m042: New Zealand vs Belgium</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">

</xml_diff>

<commit_message>
feat(auth): add password protection for participants from sheet
</commit_message>
<xml_diff>
--- a/porra_mundial_db.xlsx
+++ b/porra_mundial_db.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,6 +433,11 @@
       <c r="C1" t="inlineStr">
         <is>
           <t>paid</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>password</t>
         </is>
       </c>
     </row>
@@ -2692,7 +2697,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5489,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -23413,7 +23418,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Partido m042: New Zealand vs Belgium</t>
+          <t>Partido m100: W95 vs W96</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(events): restrict E2 random selection to group stage matches
</commit_message>
<xml_diff>
--- a/porra_mundial_db.xlsx
+++ b/porra_mundial_db.xlsx
@@ -1813,7 +1813,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -5489,7 +5489,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -23418,7 +23418,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Partido m100: W95 vs W96</t>
+          <t>Partido m025: Germany vs Curaçao</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(matches): set one random wild match per group stage matchday
</commit_message>
<xml_diff>
--- a/porra_mundial_db.xlsx
+++ b/porra_mundial_db.xlsx
@@ -1553,7 +1553,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -3945,7 +3945,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -23418,7 +23418,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Partido m025: Germany vs Curaçao</t>
+          <t>Partido m066: DR Congo vs Uzbekistan</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(excel): update spreadsheet with user-provided api_ids
</commit_message>
<xml_diff>
--- a/porra_mundial_db.xlsx
+++ b/porra_mundial_db.xlsx
@@ -478,7 +478,7 @@
       <c r="C8" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" s="0" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
@@ -14136,6 +14136,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M2" t="n">
+        <v>537327</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -14286,6 +14289,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M5" t="n">
+        <v>537330</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -14386,6 +14392,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M7" t="n">
+        <v>537332</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -14486,6 +14495,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M9" t="n">
+        <v>537334</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -14586,6 +14598,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M11" t="n">
+        <v>537336</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -14636,6 +14651,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M12" t="n">
+        <v>537337</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -14736,6 +14754,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M14" t="n">
+        <v>537339</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -14786,6 +14807,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M15" t="n">
+        <v>537340</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -14836,6 +14860,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M16" t="n">
+        <v>537342</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -14886,6 +14913,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M17" t="n">
+        <v>537341</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -14936,6 +14966,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M18" t="n">
+        <v>537343</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -14986,6 +15019,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M19" t="n">
+        <v>537344</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -15086,6 +15122,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M21" t="n">
+        <v>537346</v>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="9">
       <c r="A22" s="6" t="inlineStr">
@@ -15186,6 +15225,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M23" t="n">
+        <v>537347</v>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="9">
       <c r="A24" s="6" t="inlineStr">
@@ -15339,6 +15381,9 @@
           <t>TRUE</t>
         </is>
       </c>
+      <c r="M26" t="n">
+        <v>537351</v>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="9">
       <c r="A27" s="6" t="inlineStr">
@@ -15389,6 +15434,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M27" t="n">
+        <v>537352</v>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="9">
       <c r="A28" s="6" t="inlineStr">
@@ -15439,6 +15487,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M28" t="n">
+        <v>537353</v>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="9">
       <c r="A29" s="6" t="inlineStr">
@@ -15489,6 +15540,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M29" t="n">
+        <v>537354</v>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="9">
       <c r="A30" s="6" t="inlineStr">
@@ -15539,6 +15593,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M30" t="n">
+        <v>537356</v>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="9">
       <c r="A31" s="6" t="inlineStr">
@@ -15589,6 +15646,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M31" t="n">
+        <v>537355</v>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="9">
       <c r="A32" s="6" t="inlineStr">
@@ -15639,6 +15699,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M32" t="n">
+        <v>537357</v>
+      </c>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="9">
       <c r="A33" s="6" t="inlineStr">
@@ -15689,6 +15752,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M33" t="n">
+        <v>537358</v>
+      </c>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="9">
       <c r="A34" s="6" t="inlineStr">
@@ -15739,6 +15805,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M34" t="n">
+        <v>537359</v>
+      </c>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="9">
       <c r="A35" s="6" t="inlineStr">
@@ -15789,6 +15858,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M35" t="n">
+        <v>537360</v>
+      </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="9">
       <c r="A36" s="6" t="inlineStr">
@@ -15839,6 +15911,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M36" t="n">
+        <v>537362</v>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="9">
       <c r="A37" s="6" t="inlineStr">
@@ -15889,6 +15964,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M37" t="n">
+        <v>537361</v>
+      </c>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="9">
       <c r="A38" s="6" t="inlineStr">
@@ -15939,6 +16017,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M38" t="n">
+        <v>537363</v>
+      </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="9">
       <c r="A39" s="6" t="inlineStr">
@@ -15989,6 +16070,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M39" t="n">
+        <v>537364</v>
+      </c>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="9">
       <c r="A40" s="6" t="inlineStr">
@@ -16039,6 +16123,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M40" t="n">
+        <v>537365</v>
+      </c>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="9">
       <c r="A41" s="6" t="inlineStr">
@@ -16089,6 +16176,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M41" t="n">
+        <v>537366</v>
+      </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="9">
       <c r="A42" s="6" t="inlineStr">
@@ -16139,6 +16229,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M42" t="n">
+        <v>537368</v>
+      </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="9">
       <c r="A43" s="6" t="inlineStr">
@@ -16189,6 +16282,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M43" t="n">
+        <v>537367</v>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="9">
       <c r="A44" s="6" t="inlineStr">
@@ -16289,6 +16385,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M45" t="n">
+        <v>537370</v>
+      </c>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="9">
       <c r="A46" s="6" t="inlineStr">
@@ -16339,6 +16438,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M46" t="n">
+        <v>537371</v>
+      </c>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="9">
       <c r="A47" s="6" t="inlineStr">
@@ -16487,6 +16589,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M49" t="n">
+        <v>537373</v>
+      </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="9">
       <c r="A50" s="6" t="inlineStr">
@@ -16537,6 +16642,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M50" t="n">
+        <v>537391</v>
+      </c>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="9">
       <c r="A51" s="6" t="inlineStr">
@@ -16587,6 +16695,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M51" t="n">
+        <v>537392</v>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="9">
       <c r="A52" s="6" t="inlineStr">
@@ -16637,6 +16748,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M52" t="n">
+        <v>537393</v>
+      </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="9">
       <c r="A53" s="6" t="inlineStr">
@@ -16687,6 +16801,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M53" t="n">
+        <v>537394</v>
+      </c>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="9">
       <c r="A54" s="6" t="inlineStr">
@@ -16737,6 +16854,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M54" t="n">
+        <v>537395</v>
+      </c>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="9">
       <c r="A55" s="6" t="inlineStr">
@@ -16787,6 +16907,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M55" t="n">
+        <v>537396</v>
+      </c>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="9">
       <c r="A56" s="6" t="inlineStr">
@@ -16837,6 +16960,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M56" t="n">
+        <v>537397</v>
+      </c>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="9">
       <c r="A57" s="6" t="inlineStr">
@@ -16993,6 +17119,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M59" t="n">
+        <v>537400</v>
+      </c>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="9">
       <c r="A60" s="6" t="inlineStr">
@@ -17043,6 +17172,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M60" t="n">
+        <v>537402</v>
+      </c>
     </row>
     <row r="61" ht="15.75" customHeight="1" s="9">
       <c r="A61" s="6" t="inlineStr">
@@ -17455,6 +17587,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M68" t="n">
+        <v>537409</v>
+      </c>
     </row>
     <row r="69" ht="15.75" customHeight="1" s="9">
       <c r="A69" s="6" t="inlineStr">
@@ -17505,6 +17640,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M69" t="n">
+        <v>537410</v>
+      </c>
     </row>
     <row r="70" ht="15.75" customHeight="1" s="9">
       <c r="A70" s="6" t="inlineStr">
@@ -17555,6 +17693,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M70" t="n">
+        <v>537411</v>
+      </c>
     </row>
     <row r="71" ht="15.75" customHeight="1" s="9">
       <c r="A71" s="6" t="inlineStr">
@@ -17605,6 +17746,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M71" t="n">
+        <v>537412</v>
+      </c>
     </row>
     <row r="72" ht="15.75" customHeight="1" s="9">
       <c r="A72" s="6" t="inlineStr">
@@ -17653,6 +17797,9 @@
       <c r="L72" s="6" t="b">
         <v>1</v>
       </c>
+      <c r="M72" t="n">
+        <v>537413</v>
+      </c>
     </row>
     <row r="73" ht="15.75" customHeight="1" s="9">
       <c r="A73" s="6" t="inlineStr">
@@ -17702,6 +17849,9 @@
         <is>
           <t>FALSE</t>
         </is>
+      </c>
+      <c r="M73" t="n">
+        <v>537414</v>
       </c>
     </row>
     <row r="74" ht="15.75" customHeight="1" s="9">

</xml_diff>

<commit_message>
data(excel): update spreadsheet with all user-provided api_ids
</commit_message>
<xml_diff>
--- a/porra_mundial_db.xlsx
+++ b/porra_mundial_db.xlsx
@@ -14128,7 +14128,7 @@
       </c>
       <c r="K2" s="6" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>finished</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
@@ -14136,7 +14136,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="0" t="n">
         <v>537327</v>
       </c>
     </row>
@@ -14189,6 +14189,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M3" t="n">
+        <v>537328</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -14239,6 +14242,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M4" t="n">
+        <v>537329</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -14289,7 +14295,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="0" t="n">
         <v>537330</v>
       </c>
     </row>
@@ -14342,6 +14348,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M6" t="n">
+        <v>537331</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -14392,7 +14401,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M7" t="n">
+      <c r="M7" s="0" t="n">
         <v>537332</v>
       </c>
     </row>
@@ -14445,6 +14454,7 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -14495,7 +14505,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M9" t="n">
+      <c r="M9" s="0" t="n">
         <v>537334</v>
       </c>
     </row>
@@ -14548,6 +14558,7 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -14598,7 +14609,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M11" t="n">
+      <c r="M11" s="0" t="n">
         <v>537336</v>
       </c>
     </row>
@@ -14651,7 +14662,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M12" t="n">
+      <c r="M12" s="0" t="n">
         <v>537337</v>
       </c>
     </row>
@@ -14704,6 +14715,7 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -14754,7 +14766,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M14" t="n">
+      <c r="M14" s="0" t="n">
         <v>537339</v>
       </c>
     </row>
@@ -14807,7 +14819,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M15" t="n">
+      <c r="M15" s="0" t="n">
         <v>537340</v>
       </c>
     </row>
@@ -14860,7 +14872,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M16" t="n">
+      <c r="M16" s="0" t="n">
         <v>537342</v>
       </c>
     </row>
@@ -14913,7 +14925,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M17" t="n">
+      <c r="M17" s="0" t="n">
         <v>537341</v>
       </c>
     </row>
@@ -14966,7 +14978,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M18" t="n">
+      <c r="M18" s="0" t="n">
         <v>537343</v>
       </c>
     </row>
@@ -15019,7 +15031,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M19" t="n">
+      <c r="M19" s="0" t="n">
         <v>537344</v>
       </c>
     </row>
@@ -15072,6 +15084,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M20" t="n">
+        <v>537345</v>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="9">
       <c r="A21" s="6" t="inlineStr">
@@ -15122,7 +15137,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M21" t="n">
+      <c r="M21" s="0" t="n">
         <v>537346</v>
       </c>
     </row>
@@ -15175,6 +15190,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M22" t="n">
+        <v>537348</v>
+      </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="9">
       <c r="A23" s="6" t="inlineStr">
@@ -15225,7 +15243,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M23" t="n">
+      <c r="M23" s="0" t="n">
         <v>537347</v>
       </c>
     </row>
@@ -15278,6 +15296,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M24" t="n">
+        <v>537349</v>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="9">
       <c r="A25" s="6" t="inlineStr">
@@ -15381,7 +15402,7 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="M26" t="n">
+      <c r="M26" s="0" t="n">
         <v>537351</v>
       </c>
     </row>
@@ -15434,7 +15455,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M27" t="n">
+      <c r="M27" s="0" t="n">
         <v>537352</v>
       </c>
     </row>
@@ -15487,7 +15508,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M28" t="n">
+      <c r="M28" s="0" t="n">
         <v>537353</v>
       </c>
     </row>
@@ -15540,7 +15561,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M29" t="n">
+      <c r="M29" s="0" t="n">
         <v>537354</v>
       </c>
     </row>
@@ -15593,7 +15614,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M30" t="n">
+      <c r="M30" s="0" t="n">
         <v>537356</v>
       </c>
     </row>
@@ -15646,7 +15667,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M31" t="n">
+      <c r="M31" s="0" t="n">
         <v>537355</v>
       </c>
     </row>
@@ -15699,7 +15720,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M32" t="n">
+      <c r="M32" s="0" t="n">
         <v>537357</v>
       </c>
     </row>
@@ -15752,7 +15773,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M33" t="n">
+      <c r="M33" s="0" t="n">
         <v>537358</v>
       </c>
     </row>
@@ -15805,7 +15826,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M34" t="n">
+      <c r="M34" s="0" t="n">
         <v>537359</v>
       </c>
     </row>
@@ -15858,7 +15879,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M35" t="n">
+      <c r="M35" s="0" t="n">
         <v>537360</v>
       </c>
     </row>
@@ -15911,7 +15932,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M36" t="n">
+      <c r="M36" s="0" t="n">
         <v>537362</v>
       </c>
     </row>
@@ -15964,7 +15985,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M37" t="n">
+      <c r="M37" s="0" t="n">
         <v>537361</v>
       </c>
     </row>
@@ -16017,7 +16038,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M38" t="n">
+      <c r="M38" s="0" t="n">
         <v>537363</v>
       </c>
     </row>
@@ -16070,7 +16091,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M39" t="n">
+      <c r="M39" s="0" t="n">
         <v>537364</v>
       </c>
     </row>
@@ -16123,7 +16144,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M40" t="n">
+      <c r="M40" s="0" t="n">
         <v>537365</v>
       </c>
     </row>
@@ -16176,7 +16197,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M41" t="n">
+      <c r="M41" s="0" t="n">
         <v>537366</v>
       </c>
     </row>
@@ -16229,7 +16250,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M42" t="n">
+      <c r="M42" s="0" t="n">
         <v>537368</v>
       </c>
     </row>
@@ -16282,7 +16303,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M43" t="n">
+      <c r="M43" s="0" t="n">
         <v>537367</v>
       </c>
     </row>
@@ -16335,6 +16356,7 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="9">
       <c r="A45" s="6" t="inlineStr">
@@ -16385,7 +16407,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M45" t="n">
+      <c r="M45" s="0" t="n">
         <v>537370</v>
       </c>
     </row>
@@ -16438,7 +16460,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M46" t="n">
+      <c r="M46" s="0" t="n">
         <v>537371</v>
       </c>
     </row>
@@ -16489,6 +16511,7 @@
       <c r="L47" s="6" t="b">
         <v>1</v>
       </c>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="9">
       <c r="A48" s="6" t="inlineStr">
@@ -16539,6 +16562,7 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="9">
       <c r="A49" s="6" t="inlineStr">
@@ -16589,7 +16613,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M49" t="n">
+      <c r="M49" s="0" t="n">
         <v>537373</v>
       </c>
     </row>
@@ -16642,7 +16666,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M50" t="n">
+      <c r="M50" s="0" t="n">
         <v>537391</v>
       </c>
     </row>
@@ -16695,7 +16719,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M51" t="n">
+      <c r="M51" s="0" t="n">
         <v>537392</v>
       </c>
     </row>
@@ -16748,7 +16772,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M52" t="n">
+      <c r="M52" s="0" t="n">
         <v>537393</v>
       </c>
     </row>
@@ -16801,7 +16825,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M53" t="n">
+      <c r="M53" s="0" t="n">
         <v>537394</v>
       </c>
     </row>
@@ -16854,7 +16878,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M54" t="n">
+      <c r="M54" s="0" t="n">
         <v>537395</v>
       </c>
     </row>
@@ -16907,7 +16931,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M55" t="n">
+      <c r="M55" s="0" t="n">
         <v>537396</v>
       </c>
     </row>
@@ -16960,7 +16984,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M56" t="n">
+      <c r="M56" s="0" t="n">
         <v>537397</v>
       </c>
     </row>
@@ -17119,7 +17143,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M59" t="n">
+      <c r="M59" s="0" t="n">
         <v>537400</v>
       </c>
     </row>
@@ -17172,7 +17196,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M60" t="n">
+      <c r="M60" s="0" t="n">
         <v>537402</v>
       </c>
     </row>
@@ -17278,6 +17302,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M62" t="n">
+        <v>537403</v>
+      </c>
     </row>
     <row r="63" ht="15.75" customHeight="1" s="9">
       <c r="A63" s="6" t="inlineStr">
@@ -17434,6 +17461,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M65" t="n">
+        <v>537406</v>
+      </c>
     </row>
     <row r="66" ht="15.75" customHeight="1" s="9">
       <c r="A66" s="6" t="inlineStr">
@@ -17537,6 +17567,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="M67" t="n">
+        <v>537408</v>
+      </c>
     </row>
     <row r="68" ht="15.75" customHeight="1" s="9">
       <c r="A68" s="6" t="inlineStr">
@@ -17587,7 +17620,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M68" t="n">
+      <c r="M68" s="0" t="n">
         <v>537409</v>
       </c>
     </row>
@@ -17640,7 +17673,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M69" t="n">
+      <c r="M69" s="0" t="n">
         <v>537410</v>
       </c>
     </row>
@@ -17693,7 +17726,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M70" t="n">
+      <c r="M70" s="0" t="n">
         <v>537411</v>
       </c>
     </row>
@@ -17746,7 +17779,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M71" t="n">
+      <c r="M71" s="0" t="n">
         <v>537412</v>
       </c>
     </row>
@@ -17797,7 +17830,7 @@
       <c r="L72" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="M72" t="n">
+      <c r="M72" s="0" t="n">
         <v>537413</v>
       </c>
     </row>
@@ -17850,7 +17883,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M73" t="n">
+      <c r="M73" s="0" t="n">
         <v>537414</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data(excel): populate remaining Bosnia and Cape Verde api_ids
</commit_message>
<xml_diff>
--- a/porra_mundial_db.xlsx
+++ b/porra_mundial_db.xlsx
@@ -14189,7 +14189,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="0" t="n">
         <v>537328</v>
       </c>
     </row>
@@ -14242,7 +14242,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" s="0" t="n">
         <v>537329</v>
       </c>
     </row>
@@ -14348,7 +14348,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M6" t="n">
+      <c r="M6" s="0" t="n">
         <v>537331</v>
       </c>
     </row>
@@ -14454,7 +14454,9 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" s="0" t="n">
+        <v>537333</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -14558,7 +14560,9 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" s="0" t="n">
+        <v>537335</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -14715,7 +14719,9 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" s="0" t="n">
+        <v>537338</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -15084,7 +15090,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M20" t="n">
+      <c r="M20" s="0" t="n">
         <v>537345</v>
       </c>
     </row>
@@ -15190,7 +15196,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M22" t="n">
+      <c r="M22" s="0" t="n">
         <v>537348</v>
       </c>
     </row>
@@ -15296,7 +15302,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M24" t="n">
+      <c r="M24" s="0" t="n">
         <v>537349</v>
       </c>
     </row>
@@ -16356,7 +16362,9 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
+      <c r="M44" s="0" t="n">
+        <v>537369</v>
+      </c>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="9">
       <c r="A45" s="6" t="inlineStr">
@@ -16511,7 +16519,9 @@
       <c r="L47" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" s="0" t="n">
+        <v>537372</v>
+      </c>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="9">
       <c r="A48" s="6" t="inlineStr">
@@ -16562,7 +16572,9 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
+      <c r="M48" s="0" t="n">
+        <v>537374</v>
+      </c>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="9">
       <c r="A49" s="6" t="inlineStr">
@@ -17302,7 +17314,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M62" t="n">
+      <c r="M62" s="0" t="n">
         <v>537403</v>
       </c>
     </row>
@@ -17461,7 +17473,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M65" t="n">
+      <c r="M65" s="0" t="n">
         <v>537406</v>
       </c>
     </row>
@@ -17567,7 +17579,7 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="M67" t="n">
+      <c r="M67" s="0" t="n">
         <v>537408</v>
       </c>
     </row>

</xml_diff>